<commit_message>
DC Jack Part #
</commit_message>
<xml_diff>
--- a/Hardware/Basic/novus_t1200xe_0.8.1_pa_basic_bom_all.xlsx
+++ b/Hardware/Basic/novus_t1200xe_0.8.1_pa_basic_bom_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Home\Documents\EAGLE\Toshiba-T1200xe-PSU\jlcpcb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E02888-81C9-4340-9CC8-90B9F4CD77C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638DA643-DA22-427D-ABCC-EA4924C1D783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{8EE36123-969F-4745-9641-1E84872CB962}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8EE36123-969F-4745-9641-1E84872CB962}"/>
   </bookViews>
   <sheets>
     <sheet name="novus_t1200xe_pm_dual_d8" sheetId="1" r:id="rId1"/>
@@ -991,18 +991,9 @@
     <t>J1</t>
   </si>
   <si>
-    <t>DC-005-25A</t>
-  </si>
-  <si>
     <t>DC_Jack</t>
   </si>
   <si>
-    <t>C136715</t>
-  </si>
-  <si>
-    <t>-25℃~+80℃ 2.5mm 30V 500mA 6.4mm DC Power Jack Right Angle Plugin DC Power Connectors ROHS</t>
-  </si>
-  <si>
     <t>S2</t>
   </si>
   <si>
@@ -1016,6 +1007,15 @@
   </si>
   <si>
     <t>-40℃~+90℃ 1,000,000 cycles 12V 1N 5.85mm 50mA 6.2mm 6.2mm PC Pin Right Angle Round Button SPST-NO 弯插,6.2x6.2mm Tactile Switches ROHS</t>
+  </si>
+  <si>
+    <t>DC-005-5A-3.0</t>
+  </si>
+  <si>
+    <t>C388625</t>
+  </si>
+  <si>
+    <t>-20℃~+70℃ 24V 3mm 5A 6.2mm DC Power Jack Right Angle Plugin DC Power Connectors ROHS</t>
   </si>
 </sst>
 </file>
@@ -1505,15 +1505,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3696,7 +3693,7 @@
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="3" t="s">
+      <c r="A103" s="1" t="s">
         <v>305</v>
       </c>
       <c r="B103" s="1" t="s">
@@ -3713,7 +3710,7 @@
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="3" t="s">
+      <c r="A104" s="1" t="s">
         <v>310</v>
       </c>
       <c r="B104" s="1" t="s">
@@ -3730,7 +3727,7 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="3" t="s">
+      <c r="A105" s="1" t="s">
         <v>315</v>
       </c>
       <c r="B105" s="1" t="s">
@@ -3747,7 +3744,7 @@
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="3" t="s">
+      <c r="A106" s="1" t="s">
         <v>316</v>
       </c>
       <c r="B106" s="1" t="s">
@@ -3764,7 +3761,7 @@
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
+      <c r="A107" s="1" t="s">
         <v>320</v>
       </c>
       <c r="B107" s="1" t="s">
@@ -3781,7 +3778,7 @@
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="3" t="s">
+      <c r="A108" s="1" t="s">
         <v>321</v>
       </c>
       <c r="B108" s="1" t="s">
@@ -3798,37 +3795,37 @@
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="3" t="s">
+      <c r="A109" s="1" t="s">
         <v>322</v>
       </c>
       <c r="B109" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C109" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="C109" s="1" t="s">
+      <c r="D109" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="D109" s="1" t="s">
+      <c r="B110" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="E109" s="1" t="s">
+      <c r="C110" s="1" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="3" t="s">
+      <c r="D110" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="E110" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="C110" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="D110" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="E110" s="1" t="s">
-        <v>331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>